<commit_message>
Excel file example updated. With this file, the execution works on a virtual nodegrid manager.
</commit_message>
<xml_diff>
--- a/examples/playbooks/system-roles/Migration_Automation_Managed_Devices/Nodegrid_Importer_Template.xlsx
+++ b/examples/playbooks/system-roles/Migration_Automation_Managed_Devices/Nodegrid_Importer_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId3"/>
@@ -353,6 +353,9 @@
     <t xml:space="preserve">enable_serial_port_settings_via_escape_sequence</t>
   </si>
   <si>
+    <t xml:space="preserve">no</t>
+  </si>
+  <si>
     <t xml:space="preserve">router1</t>
   </si>
   <si>
@@ -372,9 +375,6 @@
   </si>
   <si>
     <t xml:space="preserve">enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no</t>
   </si>
   <si>
     <t xml:space="preserve">router2</t>
@@ -2629,7 +2629,7 @@
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>25</v>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>25</v>
@@ -2728,7 +2728,7 @@
     </row>
     <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>25</v>
@@ -2779,7 +2779,7 @@
     </row>
     <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>25</v>
@@ -2995,19 +2995,19 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
@@ -3017,10 +3017,10 @@
         <v>9600</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>7</v>
@@ -3029,7 +3029,7 @@
         <v>1</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P2" s="15" t="s">
         <v>55</v>
@@ -3046,15 +3046,15 @@
         <v>55</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>25</v>
@@ -3066,7 +3066,7 @@
         <v>117</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15"/>
@@ -3076,10 +3076,10 @@
         <v>9600</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>7</v>
@@ -3088,7 +3088,7 @@
         <v>1</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P3" s="15" t="s">
         <v>55</v>
@@ -3108,12 +3108,12 @@
         <v>118</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>25</v>
@@ -3125,7 +3125,7 @@
         <v>120</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
@@ -3135,10 +3135,10 @@
         <v>9600</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>7</v>
@@ -3147,7 +3147,7 @@
         <v>1</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P4" s="15" t="s">
         <v>55</v>
@@ -3164,15 +3164,15 @@
         <v>55</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W4" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>25</v>
@@ -3184,7 +3184,7 @@
         <v>122</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="15"/>
@@ -3194,10 +3194,10 @@
         <v>9600</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>7</v>
@@ -3206,7 +3206,7 @@
         <v>1</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P5" s="15" t="s">
         <v>55</v>
@@ -3226,12 +3226,12 @@
         <v>118</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>25</v>
@@ -3240,10 +3240,10 @@
         <v>123</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
@@ -3253,10 +3253,10 @@
         <v>9600</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M6" s="1" t="n">
         <v>7</v>
@@ -3265,7 +3265,7 @@
         <v>1</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P6" s="15" t="s">
         <v>55</v>
@@ -3285,7 +3285,7 @@
         <v>118</v>
       </c>
       <c r="W6" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -3457,7 +3457,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>25</v>
@@ -3483,10 +3483,10 @@
         <v>9600</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>7</v>
@@ -3495,7 +3495,7 @@
         <v>1</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P2" s="15" t="s">
         <v>55</v>
@@ -3512,16 +3512,16 @@
         <v>55</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X2" s="15"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>25</v>
@@ -3547,10 +3547,10 @@
         <v>9600</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>7</v>
@@ -3559,7 +3559,7 @@
         <v>1</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P3" s="15" t="s">
         <v>55</v>
@@ -3579,13 +3579,13 @@
         <v>118</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X3" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>25</v>
@@ -3611,10 +3611,10 @@
         <v>9600</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>7</v>
@@ -3623,7 +3623,7 @@
         <v>1</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P4" s="15" t="s">
         <v>55</v>
@@ -3640,16 +3640,16 @@
         <v>55</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="W4" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>25</v>
@@ -3675,10 +3675,10 @@
         <v>9600</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>7</v>
@@ -3687,7 +3687,7 @@
         <v>1</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P5" s="15" t="s">
         <v>55</v>
@@ -3707,7 +3707,7 @@
         <v>118</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X5" s="15"/>
     </row>
@@ -3823,7 +3823,7 @@
         <v>142</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E2" s="15" t="s">
         <v>143</v>
@@ -3852,7 +3852,7 @@
         <v>145</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E3" s="15" t="s">
         <v>143</v>
@@ -3881,7 +3881,7 @@
         <v>146</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>143</v>
@@ -3918,7 +3918,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.36"/>
@@ -4001,7 +4001,7 @@
       <c r="T1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B2" s="15" t="s">
@@ -4013,54 +4013,54 @@
       <c r="D2" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>115</v>
+      <c r="H2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="M2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="N2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="O2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="P2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="R2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="S2" s="15" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B3" s="15" t="s">
@@ -4072,19 +4072,31 @@
       <c r="D3" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>24</v>
+      <c r="A4" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>25</v>
@@ -4095,18 +4107,30 @@
       <c r="D4" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -4118,19 +4142,31 @@
       <c r="D5" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="15" t="s">
         <v>166</v>
       </c>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
     </row>
     <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>24</v>
+      <c r="A6" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>25</v>
@@ -4141,19 +4177,31 @@
       <c r="D6" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>24</v>
+      <c r="A7" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>25</v>
@@ -4164,18 +4212,30 @@
       <c r="D7" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="15" t="s">
@@ -4187,18 +4247,30 @@
       <c r="D8" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="15" t="s">
         <v>166</v>
       </c>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="15"/>
+      <c r="S8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B9" s="15" t="s">
@@ -4210,18 +4282,30 @@
       <c r="D9" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B10" s="15" t="s">
@@ -4233,19 +4317,31 @@
       <c r="D10" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>24</v>
+      <c r="A11" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>25</v>
@@ -4256,15 +4352,39 @@
       <c r="D11" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="15" t="s">
         <v>168</v>
       </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
+      <c r="O11" s="15"/>
+      <c r="P11" s="15"/>
+      <c r="Q11" s="15"/>
+      <c r="R11" s="15"/>
+      <c r="S11" s="15"/>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D15" s="15"/>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D18" s="15"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4357,7 +4477,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>55</v>
@@ -4375,16 +4495,16 @@
         <v>58</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N2" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="P2" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="P2" s="15" t="s">
-        <v>111</v>
-      </c>
       <c r="R2" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="T2" s="15" t="n">
         <v>5</v>
@@ -4393,7 +4513,7 @@
         <v>1</v>
       </c>
       <c r="X2" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Z2" s="1" t="s">
         <v>165</v>
@@ -4410,7 +4530,7 @@
         <v>128</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E3" s="15" t="s">
         <v>182</v>
@@ -4419,7 +4539,7 @@
         <v>75</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J3" s="15" t="s">
         <v>183</v>
@@ -4513,7 +4633,7 @@
         <v>8</v>
       </c>
       <c r="X5" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4832,7 +4952,7 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E43" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="L43" s="15" t="s">
         <v>267</v>

</xml_diff>

<commit_message>
Fixes: - Clean up and better Ansible tasks descriptions
</commit_message>
<xml_diff>
--- a/examples/playbooks/system-roles/Migration_Automation_Managed_Devices/Nodegrid_Importer_Template.xlsx
+++ b/examples/playbooks/system-roles/Migration_Automation_Managed_Devices/Nodegrid_Importer_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="425">
   <si>
     <t xml:space="preserve">📘 Nodegrid Template – Overview &amp; Usage Guide</t>
   </si>
@@ -71,10 +71,16 @@
     <t xml:space="preserve">Contains USB serial configurations for virtual or physical devices.</t>
   </si>
   <si>
+    <t xml:space="preserve">Device_Permissions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defines the Groups and their respective Device Access permissions.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Discovery_Rules</t>
   </si>
   <si>
-    <t xml:space="preserve">Contains Port Discovery Rules, which are required to auto detect Serial and KVM ports on appliance, for example from Vertiv, Opengear, Raritan</t>
+    <t xml:space="preserve">Contains Port Discovery Rules, which are required to auto detect Serial and KVM ports on appliance, for example from Vertiv, Opengear, Raritan.</t>
   </si>
   <si>
     <t xml:space="preserve">Update Configuration Sheets</t>
@@ -107,7 +113,7 @@
     <t xml:space="preserve">NGM-Coordinator</t>
   </si>
   <si>
-    <t xml:space="preserve">127.0.0.10</t>
+    <t xml:space="preserve">127.0.0.1</t>
   </si>
   <si>
     <t xml:space="preserve">22</t>
@@ -2080,7 +2086,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="11" t="s">
@@ -2098,8 +2104,15 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>17</v>
+      </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -2120,15 +2133,8 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
-      <c r="B14" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="12"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -2138,10 +2144,15 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="B15" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="12"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -2151,11 +2162,18 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
+    <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
@@ -2175,7 +2193,12 @@
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
     </row>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+    </row>
     <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2191,7 +2214,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2220,75 +2243,75 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F2" s="15"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>28</v>
       </c>
       <c r="F3" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>27</v>
-      </c>
       <c r="E4" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="15"/>
     </row>
@@ -2336,496 +2359,496 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J2" s="15"/>
       <c r="K2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J3" s="15"/>
       <c r="K3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M3" s="15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q3" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J4" s="15"/>
       <c r="K4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M4" s="15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N4" s="15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q4" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R4" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J5" s="15"/>
       <c r="K5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q5" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P6" s="1" t="n">
         <v>1</v>
       </c>
       <c r="Q6" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R6" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J7" s="15"/>
       <c r="K7" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P7" s="1" t="n">
         <v>2</v>
       </c>
       <c r="Q7" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M8" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q8" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R8" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F9" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G9" s="16" t="s">
-        <v>87</v>
-      </c>
       <c r="I9" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J9" s="15"/>
       <c r="K9" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O9" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P9" s="1" t="n">
         <v>1</v>
       </c>
       <c r="Q9" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R9" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J10" s="15"/>
       <c r="K10" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M10" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="P10" s="17" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Q10" s="15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R10" s="15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2924,90 +2947,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="M1" s="14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="N1" s="14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O1" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q1" s="14" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="R1" s="14" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S1" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="T1" s="14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="U1" s="14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="V1" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W1" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
@@ -3017,10 +3040,10 @@
         <v>9600</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>7</v>
@@ -3029,44 +3052,44 @@
         <v>1</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q2" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R2" s="15"/>
       <c r="S2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T2" s="15"/>
       <c r="U2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15"/>
@@ -3076,10 +3099,10 @@
         <v>9600</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>7</v>
@@ -3088,44 +3111,44 @@
         <v>1</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q3" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R3" s="15"/>
       <c r="S3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T3" s="15"/>
       <c r="U3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
@@ -3135,10 +3158,10 @@
         <v>9600</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>7</v>
@@ -3147,44 +3170,44 @@
         <v>1</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q4" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R4" s="15"/>
       <c r="S4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T4" s="15"/>
       <c r="U4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W4" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="15"/>
@@ -3194,10 +3217,10 @@
         <v>9600</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>7</v>
@@ -3206,44 +3229,44 @@
         <v>1</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q5" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R5" s="15"/>
       <c r="S5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T5" s="15"/>
       <c r="U5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
@@ -3253,10 +3276,10 @@
         <v>9600</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M6" s="1" t="n">
         <v>7</v>
@@ -3265,27 +3288,27 @@
         <v>1</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q6" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R6" s="15"/>
       <c r="S6" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T6" s="15"/>
       <c r="U6" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="W6" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -3380,102 +3403,102 @@
   <sheetData>
     <row r="1" s="15" customFormat="true" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K1" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L1" s="19" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="M1" s="19" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="N1" s="19" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O1" s="19" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="P1" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q1" s="19" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="R1" s="19" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S1" s="19" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="U1" s="19" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="V1" s="19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W1" s="19" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="X1" s="19" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="Y1" s="19" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H2" s="15"/>
       <c r="I2" s="15"/>
@@ -3483,10 +3506,10 @@
         <v>9600</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>7</v>
@@ -3495,51 +3518,51 @@
         <v>1</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q2" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R2" s="15"/>
       <c r="S2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T2" s="15"/>
       <c r="U2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="X2" s="15"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D3" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="G3" s="15" t="s">
         <v>132</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>130</v>
       </c>
       <c r="H3" s="15"/>
       <c r="I3" s="15"/>
@@ -3547,10 +3570,10 @@
         <v>9600</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>7</v>
@@ -3559,51 +3582,51 @@
         <v>1</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q3" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R3" s="15"/>
       <c r="S3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T3" s="15"/>
       <c r="U3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="X3" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="15"/>
@@ -3611,10 +3634,10 @@
         <v>9600</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>7</v>
@@ -3623,51 +3646,51 @@
         <v>1</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R4" s="15"/>
       <c r="S4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T4" s="15"/>
       <c r="U4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W4" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="X4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H5" s="15"/>
       <c r="I5" s="15"/>
@@ -3675,10 +3698,10 @@
         <v>9600</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>7</v>
@@ -3687,27 +3710,27 @@
         <v>1</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R5" s="15"/>
       <c r="S5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T5" s="15"/>
       <c r="U5" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="X5" s="15"/>
     </row>
@@ -3785,118 +3808,118 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E3" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>143</v>
-      </c>
       <c r="F3" s="15" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>144</v>
-      </c>
       <c r="G4" s="15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -3942,141 +3965,141 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="M1" s="14" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="N1" s="14" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="O1" s="14" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="Q1" s="14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R1" s="14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="S1" s="14" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="T1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="S2" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G3" s="15" t="s">
         <v>168</v>
@@ -4096,25 +4119,25 @@
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="15"/>
@@ -4131,25 +4154,25 @@
     </row>
     <row r="5" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H5" s="15"/>
       <c r="I5" s="15"/>
@@ -4166,25 +4189,25 @@
     </row>
     <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D6" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="F6" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E6" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>167</v>
-      </c>
       <c r="G6" s="15" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H6" s="15"/>
       <c r="I6" s="15"/>
@@ -4201,25 +4224,25 @@
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D7" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="G7" s="15" t="s">
         <v>170</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>168</v>
       </c>
       <c r="H7" s="15"/>
       <c r="I7" s="15"/>
@@ -4236,25 +4259,25 @@
     </row>
     <row r="8" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
@@ -4271,22 +4294,22 @@
     </row>
     <row r="9" customFormat="false" ht="17.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>168</v>
@@ -4306,22 +4329,22 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>168</v>
@@ -4341,22 +4364,22 @@
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="D11" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="E11" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>169</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>167</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>168</v>
@@ -4427,84 +4450,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="V1" s="15" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="X1" s="15" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="T2" s="15" t="n">
         <v>5</v>
@@ -4513,48 +4536,48 @@
         <v>1</v>
       </c>
       <c r="X2" s="15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N3" s="15" t="n">
         <v>9600</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="T3" s="15" t="n">
         <v>6</v>
@@ -4563,68 +4586,68 @@
         <v>2</v>
       </c>
       <c r="X3" s="15" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="AB3" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="N4" s="15" t="n">
         <v>19200</v>
       </c>
       <c r="P4" s="15" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="R4" s="15" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="T4" s="15" t="n">
         <v>7</v>
       </c>
       <c r="X4" s="15" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="N5" s="15" t="n">
         <v>57600</v>
@@ -4633,21 +4656,21 @@
         <v>8</v>
       </c>
       <c r="X5" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N6" s="15" t="n">
         <v>38400</v>
@@ -4655,13 +4678,13 @@
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="N7" s="15" t="n">
         <v>115200</v>
@@ -4669,10 +4692,10 @@
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E8" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N8" s="15" t="n">
         <v>230400</v>
@@ -4680,1021 +4703,1021 @@
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E9" s="15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E10" s="15" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="15" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="L11" s="15" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E12" s="15" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="L12" s="15" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E13" s="15" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E14" s="15" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E15" s="15" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L15" s="15" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E16" s="15" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E17" s="15" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="L17" s="15" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E18" s="15" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E19" s="15" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E20" s="15" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E21" s="15" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E22" s="15" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="L22" s="15" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E23" s="15" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="L23" s="15" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E24" s="15" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="L24" s="15" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E25" s="15" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="L25" s="15" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E26" s="15" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E27" s="15" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="L27" s="15" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E28" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L28" s="15" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E29" s="15" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="L29" s="15" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="15" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E31" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="L31" s="15" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E32" s="15" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="L32" s="15" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E33" s="15" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="L33" s="15" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E34" s="15" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="L34" s="15" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E35" s="15" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="L35" s="15" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E36" s="15" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="L36" s="15" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="15" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="L37" s="15" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E38" s="15" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L38" s="15" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E39" s="15" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="L39" s="15" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E40" s="15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L40" s="15" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E41" s="15" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="L41" s="15" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E42" s="15" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="L42" s="15" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E43" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L43" s="15" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E44" s="15" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E45" s="15" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="L45" s="15" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E46" s="15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L46" s="15" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E47" s="15" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="L47" s="15" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E48" s="15" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="L48" s="15" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E49" s="15" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="L49" s="15" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E50" s="15" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="L50" s="15" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E51" s="15" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="L51" s="15" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E52" s="15" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L52" s="15" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E53" s="15" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="L53" s="15" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E54" s="15" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="L54" s="15" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E55" s="15" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="L55" s="15" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E56" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L56" s="15" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E57" s="15" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="L57" s="15" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E58" s="15" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="L58" s="15" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E59" s="15" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="L59" s="15" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E60" s="15" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="L60" s="15" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E61" s="15" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="L61" s="15" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E62" s="15" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="L62" s="15" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E63" s="15" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="L63" s="15" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E64" s="15" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="L64" s="15" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E65" s="15" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="L65" s="15" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E66" s="15" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="L66" s="15" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L67" s="15" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L68" s="15" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L69" s="15" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L70" s="15" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L71" s="15" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L72" s="15" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L73" s="15" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L74" s="15" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L75" s="15" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L76" s="15" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L77" s="15" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L78" s="15" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L79" s="15" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L80" s="15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L81" s="15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L82" s="15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L83" s="15" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L84" s="15" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L85" s="15" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L86" s="15" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L87" s="15" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L88" s="15" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L89" s="15" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L90" s="15" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L91" s="15" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L92" s="15" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L93" s="15" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L94" s="15" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L95" s="15" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L96" s="15" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L97" s="15" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L98" s="15" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L99" s="15" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L100" s="15" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L101" s="15" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L102" s="15" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L103" s="15" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L104" s="15" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L105" s="15" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L106" s="15" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L107" s="15" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L108" s="15" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L109" s="15" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L110" s="15" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L111" s="15" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L112" s="15" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L113" s="15" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L114" s="15" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L115" s="15" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L116" s="15" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L117" s="15" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L118" s="15" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L119" s="15" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L120" s="15" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L121" s="15" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L122" s="15" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L123" s="15" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L124" s="15" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L125" s="15" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L126" s="15" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L127" s="15" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L128" s="15" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L129" s="15" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L130" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L131" s="15" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L132" s="15" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L133" s="15" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L134" s="15" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L135" s="15" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L136" s="15" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L137" s="15" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L138" s="15" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L139" s="15" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L140" s="15" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L141" s="15" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L142" s="15" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L143" s="15" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L144" s="15" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L145" s="15" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L146" s="15" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L147" s="15" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L148" s="15" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L149" s="15" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L150" s="15" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L151" s="15" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L152" s="15" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L153" s="15" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L154" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L155" s="15" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L156" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L157" s="15" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L158" s="15" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L159" s="15" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L160" s="15" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L161" s="15" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L162" s="15" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L163" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L164" s="15" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L165" s="15" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L166" s="15" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L167" s="15" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L168" s="15" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L169" s="15" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L170" s="15" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L171" s="15" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L172" s="15" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L173" s="15" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L174" s="15" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L175" s="15" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L176" s="15" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L177" s="15" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Managed Devices import fixes: - Support Managed Devices -> management - Extend the library to add support for Managed Devices Rebounce, i.e., disable a managed device, then re-enable it - Test the Managed devices 'IP Devices' SSH shared key - Update the 'Nodegrid_Importer_Template.xlsx' example template
</commit_message>
<xml_diff>
--- a/examples/playbooks/system-roles/Migration_Automation_Managed_Devices/Nodegrid_Importer_Template.xlsx
+++ b/examples/playbooks/system-roles/Migration_Automation_Managed_Devices/Nodegrid_Importer_Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="443">
   <si>
     <t xml:space="preserve">📘 Nodegrid Template – Overview &amp; Usage Guide</t>
   </si>
@@ -158,6 +158,9 @@
     <t xml:space="preserve">username</t>
   </si>
   <si>
+    <t xml:space="preserve">credential</t>
+  </si>
+  <si>
     <t xml:space="preserve">password</t>
   </si>
   <si>
@@ -179,6 +182,30 @@
     <t xml:space="preserve">port_number</t>
   </si>
   <si>
+    <t xml:space="preserve">allow_ssh_protocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ssh_port</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allow_pre-shared_ssh_key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ssh_key_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ssh_private_key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ssh_public_key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mgmt_discover_ports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rebounce</t>
+  </si>
+  <si>
     <t xml:space="preserve">cf_Rack_Location</t>
   </si>
   <si>
@@ -581,6 +608,12 @@
     <t xml:space="preserve">128technology.png</t>
   </si>
   <si>
+    <t xml:space="preserve">ask_during_login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ecdsa_256</t>
+  </si>
+  <si>
     <t xml:space="preserve">air_flow-temperature.png</t>
   </si>
   <si>
@@ -605,6 +638,12 @@
     <t xml:space="preserve">door_status</t>
   </si>
   <si>
+    <t xml:space="preserve">set_now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ecdsa_384</t>
+  </si>
+  <si>
     <t xml:space="preserve">apc.png</t>
   </si>
   <si>
@@ -620,25 +659,40 @@
     <t xml:space="preserve">DCD</t>
   </si>
   <si>
+    <t xml:space="preserve">ecdsa_521</t>
+  </si>
+  <si>
     <t xml:space="preserve">device_console</t>
   </si>
   <si>
     <t xml:space="preserve">apple_black.png</t>
   </si>
   <si>
+    <t xml:space="preserve">ed25519</t>
+  </si>
+  <si>
     <t xml:space="preserve">arista.png</t>
   </si>
   <si>
     <t xml:space="preserve">ttyS5</t>
   </si>
   <si>
+    <t xml:space="preserve">rsa_1024</t>
+  </si>
+  <si>
     <t xml:space="preserve">aruba.png</t>
   </si>
   <si>
     <t xml:space="preserve">ttyS6</t>
   </si>
   <si>
+    <t xml:space="preserve">rsa_2048</t>
+  </si>
+  <si>
     <t xml:space="preserve">ttyS7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rsa_4096</t>
   </si>
   <si>
     <t xml:space="preserve">ttyS8</t>
@@ -1640,9 +1694,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="local_ip" displayName="local_ip" ref="A1:R12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:R12"/>
-  <tableColumns count="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="local_ip" displayName="local_ip" ref="A1:AA12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:AA12"/>
+  <tableColumns count="27">
     <tableColumn id="1" name="Export"/>
     <tableColumn id="2" name="ansible_inventory_name"/>
     <tableColumn id="3" name="name"/>
@@ -1652,15 +1706,24 @@
     <tableColumn id="7" name="ip_address"/>
     <tableColumn id="8" name="port"/>
     <tableColumn id="9" name="username"/>
-    <tableColumn id="10" name="password"/>
-    <tableColumn id="11" name="enable_device_state_detection_based_on_network_traffic"/>
-    <tableColumn id="12" name="multisession"/>
-    <tableColumn id="13" name="icon"/>
-    <tableColumn id="14" name="mode"/>
-    <tableColumn id="15" name="end_point"/>
-    <tableColumn id="16" name="port_number"/>
-    <tableColumn id="17" name="cf_Rack_Location"/>
-    <tableColumn id="18" name="cf_custom_field2"/>
+    <tableColumn id="10" name="credential"/>
+    <tableColumn id="11" name="password"/>
+    <tableColumn id="12" name="enable_device_state_detection_based_on_network_traffic"/>
+    <tableColumn id="13" name="multisession"/>
+    <tableColumn id="14" name="icon"/>
+    <tableColumn id="15" name="mode"/>
+    <tableColumn id="16" name="end_point"/>
+    <tableColumn id="17" name="port_number"/>
+    <tableColumn id="18" name="allow_ssh_protocol"/>
+    <tableColumn id="19" name="ssh_port"/>
+    <tableColumn id="20" name="allow_pre-shared_ssh_key"/>
+    <tableColumn id="21" name="ssh_key_type"/>
+    <tableColumn id="22" name="ssh_private_key"/>
+    <tableColumn id="23" name="ssh_public_key"/>
+    <tableColumn id="24" name="mgmt_discover_ports"/>
+    <tableColumn id="25" name="rebounce"/>
+    <tableColumn id="26" name="cf_Rack_Location"/>
+    <tableColumn id="27" name="cf_custom_field2"/>
   </tableColumns>
 </table>
 </file>
@@ -2335,7 +2398,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.33"/>
@@ -2347,14 +2410,23 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="10.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="17.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="15" width="15.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="12.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="11.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="15" width="17.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="17.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="15" width="17.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="33.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="37.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="17.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="15" width="22.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="15" width="9.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="1" width="17.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2412,6 +2484,33 @@
       <c r="R1" s="14" t="s">
         <v>51</v>
       </c>
+      <c r="S1" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="T1" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="U1" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="V1" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="W1" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="X1" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y1" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA1" s="14" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
@@ -2421,42 +2520,42 @@
         <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K2" s="15"/>
       <c r="L2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q2" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="R2" s="15" t="s">
-        <v>62</v>
+        <v>68</v>
+      </c>
+      <c r="P2" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z2" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA2" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2467,42 +2566,42 @@
         <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K3" s="15"/>
       <c r="L3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M3" s="15" t="s">
         <v>66</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q3" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R3" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
+      </c>
+      <c r="P3" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z3" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA3" s="15" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2513,45 +2612,45 @@
         <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K4" s="15"/>
       <c r="L4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M4" s="15" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="N4" s="15" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q4" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>68</v>
+      </c>
+      <c r="P4" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z4" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA4" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
         <v>26</v>
       </c>
@@ -2559,47 +2658,47 @@
         <v>27</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K5" s="15"/>
       <c r="L5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M5" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="N5" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="O5" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="P5" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z5" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="N5" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="O5" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q5" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R5" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AA5" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
         <v>26</v>
       </c>
@@ -2607,50 +2706,50 @@
         <v>27</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K6" s="15"/>
       <c r="L6" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="P6" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="P6" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R6" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z6" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA6" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
         <v>31</v>
       </c>
@@ -2658,50 +2757,50 @@
         <v>27</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E7" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>75</v>
-      </c>
       <c r="I7" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K7" s="15"/>
       <c r="L7" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="P7" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="P7" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="Q7" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R7" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z7" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA7" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
         <v>31</v>
       </c>
@@ -2709,47 +2808,47 @@
         <v>27</v>
       </c>
       <c r="C8" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="N8" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="L8" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="M8" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="N8" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="O8" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q8" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R8" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P8" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z8" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA8" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
         <v>31</v>
       </c>
@@ -2757,50 +2856,50 @@
         <v>27</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F9" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="N9" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="O9" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="P9" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="G9" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="I9" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="L9" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="M9" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="N9" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="O9" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="P9" s="1" t="n">
+      <c r="Q9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q9" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="R9" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z9" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA9" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
         <v>31</v>
       </c>
@@ -2808,74 +2907,81 @@
         <v>27</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15" t="s">
-        <v>57</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K10" s="15"/>
       <c r="L10" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M10" s="15" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="P10" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q10" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="R10" s="15" t="s">
-        <v>67</v>
+        <v>86</v>
+      </c>
+      <c r="P10" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q10" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="S10" s="17"/>
+      <c r="V10" s="17"/>
+      <c r="W10" s="17"/>
+      <c r="Z10" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="AA10" s="15" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15"/>
       <c r="D11" s="15"/>
-      <c r="K11" s="15"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
       <c r="N11" s="15"/>
       <c r="O11" s="15"/>
+      <c r="P11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15"/>
       <c r="D12" s="15"/>
-      <c r="K12" s="15"/>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
       <c r="N12" s="15"/>
       <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="11">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="R2:R1010 T2:T1010 X2:Y1010" type="list">
+      <formula1>Lookup_Table!$C$2:$C$3</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H2:H12" type="whole">
       <formula1>1</formula1>
       <formula2>65500</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="P2:P9 P11:P12" type="whole">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="Q2:Q9 S2:S9 V2:W9 Q11:Q12 S11:S12 V11:W12" type="whole">
       <formula1>1</formula1>
       <formula2>96</formula2>
     </dataValidation>
@@ -2887,20 +2993,28 @@
       <formula1>Lookup_Table!$A$2:$A$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A2:A12 K2:L12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A2:A12 L2:M12" type="list">
       <formula1>Lookup_Table!$C$2:$C$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="M2:M12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="N2:N12" type="list">
       <formula1>Lookup_Table!$E$2:$E$202</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="N2:N12" type="list">
-      <formula1>Lookup_Table!$G$2:$G$3</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="P2:P12" type="list">
+      <formula1>Lookup_Table!$J$2:$J$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="O2:O12" type="list">
-      <formula1>Lookup_Table!$J$2:$J$6</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:J1010" type="list">
+      <formula1>Lookup_Table!$AD$2:$AD$3</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="O2:O1010" type="list">
+      <formula1>Lookup_Table!$G$2:$G$4</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="U2:U1010" type="list">
+      <formula1>Lookup_Table!$AF$2:$AF$8</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2956,7 +3070,7 @@
         <v>36</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>37</v>
@@ -2971,66 +3085,66 @@
         <v>42</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="M1" s="14" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="N1" s="14" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="O1" s="14" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="Q1" s="14" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="R1" s="14" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="S1" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="T1" s="14" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="U1" s="14" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="V1" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W1" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
@@ -3040,10 +3154,10 @@
         <v>9600</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>7</v>
@@ -3052,44 +3166,44 @@
         <v>1</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q2" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R2" s="15"/>
       <c r="S2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T2" s="15"/>
       <c r="U2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15"/>
@@ -3099,10 +3213,10 @@
         <v>9600</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>7</v>
@@ -3111,44 +3225,44 @@
         <v>1</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q3" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R3" s="15"/>
       <c r="S3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T3" s="15"/>
       <c r="U3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="D4" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>122</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>113</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
@@ -3158,10 +3272,10 @@
         <v>9600</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>7</v>
@@ -3170,44 +3284,44 @@
         <v>1</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q4" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R4" s="15"/>
       <c r="S4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T4" s="15"/>
       <c r="U4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="W4" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="15"/>
@@ -3217,10 +3331,10 @@
         <v>9600</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>7</v>
@@ -3229,44 +3343,44 @@
         <v>1</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q5" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R5" s="15"/>
       <c r="S5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T5" s="15"/>
       <c r="U5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
@@ -3276,10 +3390,10 @@
         <v>9600</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M6" s="1" t="n">
         <v>7</v>
@@ -3288,27 +3402,27 @@
         <v>1</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q6" s="15" t="n">
         <v>3</v>
       </c>
       <c r="R6" s="15"/>
       <c r="S6" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T6" s="15"/>
       <c r="U6" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="W6" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -3412,7 +3526,7 @@
         <v>36</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="E1" s="18" t="s">
         <v>37</v>
@@ -3427,78 +3541,78 @@
         <v>42</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="K1" s="19" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="L1" s="19" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="M1" s="19" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="N1" s="19" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="O1" s="19" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="P1" s="19" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="Q1" s="19" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="R1" s="19" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="S1" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="U1" s="19" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="V1" s="19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W1" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="X1" s="19" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="Y1" s="19" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B2" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="H2" s="15"/>
       <c r="I2" s="15"/>
@@ -3506,10 +3620,10 @@
         <v>9600</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>7</v>
@@ -3518,51 +3632,51 @@
         <v>1</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q2" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R2" s="15"/>
       <c r="S2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T2" s="15"/>
       <c r="U2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="X2" s="15"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="H3" s="15"/>
       <c r="I3" s="15"/>
@@ -3570,10 +3684,10 @@
         <v>9600</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>7</v>
@@ -3582,51 +3696,51 @@
         <v>1</v>
       </c>
       <c r="O3" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q3" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R3" s="15"/>
       <c r="S3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T3" s="15"/>
       <c r="U3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="X3" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="15"/>
@@ -3634,10 +3748,10 @@
         <v>9600</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>7</v>
@@ -3646,51 +3760,51 @@
         <v>1</v>
       </c>
       <c r="O4" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R4" s="15"/>
       <c r="S4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T4" s="15"/>
       <c r="U4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="W4" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="X4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="H5" s="15"/>
       <c r="I5" s="15"/>
@@ -3698,10 +3812,10 @@
         <v>9600</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>7</v>
@@ -3710,27 +3824,27 @@
         <v>1</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="Q5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="R5" s="15"/>
       <c r="S5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="T5" s="15"/>
       <c r="U5" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="X5" s="15"/>
     </row>
@@ -3814,25 +3928,25 @@
         <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3843,25 +3957,25 @@
         <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3872,25 +3986,25 @@
         <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3901,25 +4015,25 @@
         <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3971,55 +4085,55 @@
         <v>21</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="M1" s="14" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="N1" s="14" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="O1" s="14" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="Q1" s="14" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="R1" s="14" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="S1" s="14" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="T1" s="14"/>
     </row>
@@ -4031,55 +4145,55 @@
         <v>27</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="M2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="S2" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,19 +4204,19 @@
         <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H3" s="15"/>
       <c r="I3" s="15"/>
@@ -4125,19 +4239,19 @@
         <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="H4" s="15"/>
       <c r="I4" s="15"/>
@@ -4160,19 +4274,19 @@
         <v>27</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H5" s="15"/>
       <c r="I5" s="15"/>
@@ -4195,19 +4309,19 @@
         <v>27</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="H6" s="15"/>
       <c r="I6" s="15"/>
@@ -4230,19 +4344,19 @@
         <v>27</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="H7" s="15"/>
       <c r="I7" s="15"/>
@@ -4265,19 +4379,19 @@
         <v>27</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
@@ -4300,19 +4414,19 @@
         <v>27</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H9" s="15"/>
       <c r="I9" s="15"/>
@@ -4335,19 +4449,19 @@
         <v>27</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H10" s="15"/>
       <c r="I10" s="15"/>
@@ -4370,19 +4484,19 @@
         <v>27</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H11" s="15"/>
       <c r="I11" s="15"/>
@@ -4426,7 +4540,7 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB177"/>
+  <dimension ref="A1:AF177"/>
   <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="15" width="21.5"/>
@@ -4446,6 +4560,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="2.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="13.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="12.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="2.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="3"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4453,81 +4569,87 @@
         <v>37</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="V1" s="15" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="X1" s="15" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>153</v>
+        <v>162</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF1" s="0" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="L2" s="15" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="T2" s="15" t="n">
         <v>5</v>
@@ -4536,48 +4658,54 @@
         <v>1</v>
       </c>
       <c r="X2" s="15" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>170</v>
+        <v>179</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="AF2" s="0" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="N3" s="15" t="n">
         <v>9600</v>
       </c>
       <c r="P3" s="15" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="T3" s="15" t="n">
         <v>6</v>
@@ -4586,68 +4714,83 @@
         <v>2</v>
       </c>
       <c r="X3" s="15" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="AB3" s="1" t="s">
-        <v>191</v>
+        <v>202</v>
+      </c>
+      <c r="AD3" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="AF3" s="0" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>192</v>
+        <v>205</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>86</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="N4" s="15" t="n">
         <v>19200</v>
       </c>
       <c r="P4" s="15" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="R4" s="15" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="T4" s="15" t="n">
         <v>7</v>
       </c>
       <c r="X4" s="15" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>168</v>
+        <v>177</v>
+      </c>
+      <c r="AF4" s="0" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="N5" s="15" t="n">
         <v>57600</v>
@@ -4656,1068 +4799,1080 @@
         <v>8</v>
       </c>
       <c r="X5" s="15" t="s">
-        <v>114</v>
+        <v>123</v>
+      </c>
+      <c r="AF5" s="0" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="N6" s="15" t="n">
         <v>38400</v>
       </c>
+      <c r="AF6" s="0" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
       <c r="N7" s="15" t="n">
         <v>115200</v>
       </c>
+      <c r="AF7" s="0" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E8" s="15" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
       <c r="N8" s="15" t="n">
         <v>230400</v>
       </c>
+      <c r="AF8" s="0" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E9" s="15" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E10" s="15" t="s">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="L10" s="15" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="15" t="s">
-        <v>207</v>
+        <v>225</v>
       </c>
       <c r="L11" s="15" t="s">
-        <v>208</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E12" s="15" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="L12" s="15" t="s">
-        <v>210</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E13" s="15" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E14" s="15" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>214</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E15" s="15" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
       <c r="L15" s="15" t="s">
-        <v>216</v>
+        <v>234</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E16" s="15" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E17" s="15" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="L17" s="15" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E18" s="15" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E19" s="15" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E20" s="15" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>226</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E21" s="15" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E22" s="15" t="s">
-        <v>229</v>
+        <v>247</v>
       </c>
       <c r="L22" s="15" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E23" s="15" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="L23" s="15" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E24" s="15" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="L24" s="15" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E25" s="15" t="s">
-        <v>235</v>
+        <v>253</v>
       </c>
       <c r="L25" s="15" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E26" s="15" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E27" s="15" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
       <c r="L27" s="15" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E28" s="15" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="L28" s="15" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E29" s="15" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="L29" s="15" t="s">
-        <v>243</v>
+        <v>261</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="15" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E31" s="15" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="L31" s="15" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E32" s="15" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="L32" s="15" t="s">
-        <v>249</v>
+        <v>267</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E33" s="15" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="L33" s="15" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E34" s="15" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
       <c r="L34" s="15" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E35" s="15" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="L35" s="15" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E36" s="15" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="L36" s="15" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="15" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="L37" s="15" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E38" s="15" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="L38" s="15" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E39" s="15" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
       <c r="L39" s="15" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E40" s="15" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="L40" s="15" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E41" s="15" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="L41" s="15" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E42" s="15" t="s">
-        <v>267</v>
+        <v>285</v>
       </c>
       <c r="L42" s="15" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E43" s="15" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="L43" s="15" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E44" s="15" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E45" s="15" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="L45" s="15" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E46" s="15" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="L46" s="15" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E47" s="15" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="L47" s="15" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E48" s="15" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="L48" s="15" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E49" s="15" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
       <c r="L49" s="15" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E50" s="15" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="L50" s="15" t="s">
-        <v>282</v>
+        <v>300</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E51" s="15" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="L51" s="15" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E52" s="15" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
       <c r="L52" s="15" t="s">
-        <v>286</v>
+        <v>304</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E53" s="15" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="L53" s="15" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E54" s="15" t="s">
-        <v>289</v>
+        <v>307</v>
       </c>
       <c r="L54" s="15" t="s">
-        <v>290</v>
+        <v>308</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E55" s="15" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
       <c r="L55" s="15" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E56" s="15" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="L56" s="15" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E57" s="15" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="L57" s="15" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E58" s="15" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="L58" s="15" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E59" s="15" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="L59" s="15" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E60" s="15" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="L60" s="15" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E61" s="15" t="s">
-        <v>302</v>
+        <v>320</v>
       </c>
       <c r="L61" s="15" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E62" s="15" t="s">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="L62" s="15" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E63" s="15" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="L63" s="15" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E64" s="15" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
       <c r="L64" s="15" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E65" s="15" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="L65" s="15" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E66" s="15" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="L66" s="15" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L67" s="15" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L68" s="15" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L69" s="15" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L70" s="15" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L71" s="15" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L72" s="15" t="s">
-        <v>319</v>
+        <v>337</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L73" s="15" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L74" s="15" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L75" s="15" t="s">
-        <v>322</v>
+        <v>340</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L76" s="15" t="s">
-        <v>323</v>
+        <v>341</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L77" s="15" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L78" s="15" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L79" s="15" t="s">
-        <v>326</v>
+        <v>344</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L80" s="15" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L81" s="15" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L82" s="15" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L83" s="15" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L84" s="15" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L85" s="15" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L86" s="15" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L87" s="15" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L88" s="15" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L89" s="15" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L90" s="15" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L91" s="15" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L92" s="15" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L93" s="15" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L94" s="15" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L95" s="15" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L96" s="15" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L97" s="15" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L98" s="15" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L99" s="15" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L100" s="15" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L101" s="15" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L102" s="15" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L103" s="15" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L104" s="15" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L105" s="15" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L106" s="15" t="s">
-        <v>353</v>
+        <v>371</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L107" s="15" t="s">
-        <v>354</v>
+        <v>372</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L108" s="15" t="s">
-        <v>355</v>
+        <v>373</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L109" s="15" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L110" s="15" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L111" s="15" t="s">
-        <v>358</v>
+        <v>376</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L112" s="15" t="s">
-        <v>359</v>
+        <v>377</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L113" s="15" t="s">
-        <v>360</v>
+        <v>378</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L114" s="15" t="s">
-        <v>361</v>
+        <v>379</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L115" s="15" t="s">
-        <v>362</v>
+        <v>380</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L116" s="15" t="s">
-        <v>363</v>
+        <v>381</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L117" s="15" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L118" s="15" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L119" s="15" t="s">
-        <v>366</v>
+        <v>384</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L120" s="15" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L121" s="15" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L122" s="15" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L123" s="15" t="s">
-        <v>370</v>
+        <v>388</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L124" s="15" t="s">
-        <v>371</v>
+        <v>389</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L125" s="15" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L126" s="15" t="s">
-        <v>373</v>
+        <v>391</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L127" s="15" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L128" s="15" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L129" s="15" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L130" s="15" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L131" s="15" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L132" s="15" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L133" s="15" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L134" s="15" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L135" s="15" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L136" s="15" t="s">
-        <v>383</v>
+        <v>401</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L137" s="15" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L138" s="15" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L139" s="15" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L140" s="15" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L141" s="15" t="s">
-        <v>388</v>
+        <v>406</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L142" s="15" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L143" s="15" t="s">
-        <v>390</v>
+        <v>408</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L144" s="15" t="s">
-        <v>391</v>
+        <v>409</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L145" s="15" t="s">
-        <v>392</v>
+        <v>410</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L146" s="15" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L147" s="15" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L148" s="15" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L149" s="15" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L150" s="15" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L151" s="15" t="s">
-        <v>398</v>
+        <v>416</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L152" s="15" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L153" s="15" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L154" s="15" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L155" s="15" t="s">
-        <v>402</v>
+        <v>420</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L156" s="15" t="s">
-        <v>403</v>
+        <v>421</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L157" s="15" t="s">
-        <v>404</v>
+        <v>422</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L158" s="15" t="s">
-        <v>405</v>
+        <v>423</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L159" s="15" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L160" s="15" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L161" s="15" t="s">
-        <v>408</v>
+        <v>426</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L162" s="15" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L163" s="15" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L164" s="15" t="s">
-        <v>411</v>
+        <v>429</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L165" s="15" t="s">
-        <v>412</v>
+        <v>430</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L166" s="15" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L167" s="15" t="s">
-        <v>414</v>
+        <v>432</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L168" s="15" t="s">
-        <v>415</v>
+        <v>433</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L169" s="15" t="s">
-        <v>416</v>
+        <v>434</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L170" s="15" t="s">
-        <v>417</v>
+        <v>435</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L171" s="15" t="s">
-        <v>418</v>
+        <v>436</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L172" s="15" t="s">
-        <v>419</v>
+        <v>437</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L173" s="15" t="s">
-        <v>420</v>
+        <v>438</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L174" s="15" t="s">
-        <v>421</v>
+        <v>439</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L175" s="15" t="s">
-        <v>422</v>
+        <v>440</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L176" s="15" t="s">
-        <v>423</v>
+        <v>441</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="L177" s="15" t="s">
-        <v>424</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>